<commit_message>
agregacion de imagenes dediferentes etapas, perdidas y estabilidad de entrenamiento
</commit_message>
<xml_diff>
--- a/PROYECTO3_requisitos.xlsx
+++ b/PROYECTO3_requisitos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unaledu-my.sharepoint.com/personal/mzueta_unal_edu_co/Documents/2025-02/Intro IA/Practica 3/practica_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_9F425ECB97D9AECF8A160B63BB9D05477634D4C7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97C268AB-EFD9-4EA5-BC33-1548C731A751}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_9F425ECB97D9AECF8A160B63BB9D05477634D4C7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88BD74CD-26DA-486B-9018-FDE645F8A0BF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -253,7 +253,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -568,10 +568,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" customWidth="1"/>
     <col min="3" max="3" width="71.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>